<commit_message>
Added one more day
</commit_message>
<xml_diff>
--- a/DCP_dataset.xlsx
+++ b/DCP_dataset.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcelasalomonipoli/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcelasalomonipoli/DCP_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D09A74-C509-2F49-BF42-D5E4A9CD7BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9881140-2997-4A43-9D1B-34D71F3AD908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="17140" xr2:uid="{EBB68BE6-B990-BB47-B7F8-0C8704CAA63B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
   <si>
     <t>N</t>
   </si>
@@ -84,6 +84,15 @@
   </si>
   <si>
     <t xml:space="preserve">Late </t>
+  </si>
+  <si>
+    <t xml:space="preserve">University </t>
+  </si>
+  <si>
+    <t>KFC, porridge</t>
+  </si>
+  <si>
+    <t>Energized</t>
   </si>
 </sst>
 </file>
@@ -341,7 +350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8473CA99-5C76-E747-83A9-8B8766DC4343}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -418,6 +427,38 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
+        <v>46315</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.8125</v>
+      </c>
+      <c r="E3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J3" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Added new data, changed Meal column contents for usability
</commit_message>
<xml_diff>
--- a/DCP_dataset.xlsx
+++ b/DCP_dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcelasalomonipoli/DCP_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0EEC5C9-754B-FA4C-A724-C109521B267E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25AD3EB4-6C0A-AC47-BBE3-D098DADAB87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="680" windowWidth="28040" windowHeight="17140" xr2:uid="{EBB68BE6-B990-BB47-B7F8-0C8704CAA63B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="23">
   <si>
     <t>N</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Caffeine at night</t>
   </si>
   <si>
-    <t>Bagels, porridge</t>
-  </si>
-  <si>
     <t>Snooze</t>
   </si>
   <si>
@@ -83,36 +80,21 @@
     <t xml:space="preserve">University </t>
   </si>
   <si>
-    <t>KFC, porridge</t>
-  </si>
-  <si>
     <t>Energized</t>
   </si>
   <si>
     <t>Free</t>
   </si>
   <si>
-    <t>Chicken pasta</t>
-  </si>
-  <si>
-    <t>Bolognese pasta</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sleepy </t>
   </si>
   <si>
-    <t>Fajitas</t>
-  </si>
-  <si>
     <t xml:space="preserve">Y </t>
   </si>
   <si>
     <t xml:space="preserve">Free </t>
   </si>
   <si>
-    <t>Burrito Bowl</t>
-  </si>
-  <si>
     <t>Meal Time</t>
   </si>
   <si>
@@ -120,6 +102,12 @@
   </si>
   <si>
     <t xml:space="preserve">N </t>
+  </si>
+  <si>
+    <t>Healthy</t>
+  </si>
+  <si>
+    <t>Fast food</t>
   </si>
 </sst>
 </file>
@@ -377,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8473CA99-5C76-E747-83A9-8B8766DC4343}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -398,28 +386,28 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E1" t="s">
         <v>5</v>
       </c>
       <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" t="s">
-        <v>10</v>
-      </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -430,7 +418,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D2" s="3">
         <v>0</v>
@@ -445,7 +433,7 @@
         <v>0.44444444444444442</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I2" t="s">
         <v>1</v>
@@ -459,10 +447,10 @@
         <v>46315</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D3" s="3">
         <v>0.8125</v>
@@ -477,7 +465,7 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I3" t="s">
         <v>1</v>
@@ -491,10 +479,10 @@
         <v>46316</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D4" s="3">
         <v>0.875</v>
@@ -509,7 +497,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="H4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I4" t="s">
         <v>1</v>
@@ -526,7 +514,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D5" s="3">
         <v>0.91666666666666663</v>
@@ -541,7 +529,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="H5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I5" t="s">
         <v>1</v>
@@ -558,7 +546,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="3">
         <v>0.95833333333333337</v>
@@ -573,10 +561,10 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="H6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="J6" t="s">
         <v>1</v>
@@ -587,16 +575,16 @@
         <v>46319</v>
       </c>
       <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>22</v>
-      </c>
-      <c r="C7" t="s">
-        <v>23</v>
       </c>
       <c r="D7" s="3">
         <v>0.91666666666666663</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F7" s="3">
         <v>6.25E-2</v>
@@ -605,13 +593,77 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="H7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I7" t="s">
         <v>1</v>
       </c>
       <c r="J7" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>46320</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0.375</v>
+      </c>
+      <c r="H8" t="s">
+        <v>10</v>
+      </c>
+      <c r="I8" t="s">
+        <v>0</v>
+      </c>
+      <c r="J8" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>46321</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="E9" t="s">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0.375</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" t="s">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>